<commit_message>
Habilitar filtro por periodo en reporte por movimientos. Guardar archivo excel con imagenes en plantilla. Generar reporte en PDF.
</commit_message>
<xml_diff>
--- a/rh/reportes/archivos/PLANTILLA FORMATO AVISO DE BAJA.xlsx
+++ b/rh/reportes/archivos/PLANTILLA FORMATO AVISO DE BAJA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gerardo\Documents\INAES\repositorio\SIA_V2\rh\reportes\archivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2D6A02-F6EA-4B47-8D8C-BDD0A2555B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF741C2-D95D-4EA7-A111-8891924F5098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2955" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVISO_DE_BAJA" sheetId="1" r:id="rId1"/>
@@ -166,46 +166,46 @@
     <t>NOMBRE DEL DIRECTOR</t>
   </si>
   <si>
-    <t>%FOLIO%</t>
-  </si>
-  <si>
-    <t>%APPATERNO%</t>
-  </si>
-  <si>
-    <t>%APMATERNO%</t>
-  </si>
-  <si>
-    <t>%NOMBRE%</t>
-  </si>
-  <si>
-    <t>%RFC%</t>
-  </si>
-  <si>
-    <t>%CLAVEPRESUPUESTAL%</t>
-  </si>
-  <si>
-    <t>%NIVEL%</t>
-  </si>
-  <si>
-    <t>%CAUSABAJA%</t>
-  </si>
-  <si>
-    <t>%NUMEMPLEADO%</t>
-  </si>
-  <si>
-    <t>%CC%</t>
-  </si>
-  <si>
-    <t>%TIPOPLAZA%</t>
-  </si>
-  <si>
-    <t>%CURP%</t>
-  </si>
-  <si>
-    <t>%ADSCRIPCION%</t>
-  </si>
-  <si>
-    <t>%FECHABAJA%</t>
+    <t>FOLIO_D</t>
+  </si>
+  <si>
+    <t>APPATERNO_D</t>
+  </si>
+  <si>
+    <t>APMATERNO_D</t>
+  </si>
+  <si>
+    <t>RFC_D</t>
+  </si>
+  <si>
+    <t>NOMBRE_D</t>
+  </si>
+  <si>
+    <t>CLAVEPRESUPUESTAL_D</t>
+  </si>
+  <si>
+    <t>NIVEL_D</t>
+  </si>
+  <si>
+    <t>CAUSABAJA_D</t>
+  </si>
+  <si>
+    <t>NUMEMPLEADO_D</t>
+  </si>
+  <si>
+    <t>CC_D</t>
+  </si>
+  <si>
+    <t>TIPOPLAZA_D</t>
+  </si>
+  <si>
+    <t>CURP_D</t>
+  </si>
+  <si>
+    <t>ADSCRIPCION_D</t>
+  </si>
+  <si>
+    <t>FECHABAJA_D</t>
   </si>
 </sst>
 </file>
@@ -704,6 +704,60 @@
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -743,65 +797,11 @@
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2997,76 +2997,76 @@
     </row>
     <row r="6" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9"/>
-      <c r="B6" s="70" t="s">
+      <c r="B6" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="70"/>
-      <c r="D6" s="70"/>
-      <c r="E6" s="70"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="70"/>
-      <c r="H6" s="70"/>
-      <c r="I6" s="70"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
       <c r="J6" s="9"/>
     </row>
     <row r="7" spans="1:12" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="71" t="s">
+      <c r="B7" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="71"/>
-      <c r="D7" s="71"/>
-      <c r="E7" s="71"/>
-      <c r="F7" s="71"/>
-      <c r="G7" s="71"/>
-      <c r="H7" s="71"/>
-      <c r="I7" s="71"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="45"/>
+      <c r="G7" s="45"/>
+      <c r="H7" s="45"/>
+      <c r="I7" s="45"/>
     </row>
     <row r="8" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="72" t="s">
+      <c r="B8" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="72"/>
-      <c r="D8" s="72"/>
-      <c r="E8" s="72"/>
-      <c r="F8" s="72"/>
-      <c r="G8" s="72"/>
-      <c r="H8" s="72"/>
-      <c r="I8" s="72"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="46"/>
+      <c r="I8" s="46"/>
     </row>
     <row r="9" spans="1:12" s="10" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="73" t="s">
+      <c r="B9" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="73"/>
-      <c r="D9" s="73"/>
-      <c r="E9" s="73" t="s">
+      <c r="C9" s="47"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="F9" s="73"/>
-      <c r="G9" s="74" t="s">
+      <c r="F9" s="47"/>
+      <c r="G9" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="H9" s="75"/>
-      <c r="I9" s="76"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="50"/>
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="62"/>
-      <c r="D10" s="63"/>
-      <c r="E10" s="64" t="s">
+      <c r="C10" s="52"/>
+      <c r="D10" s="53"/>
+      <c r="E10" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="F10" s="65"/>
-      <c r="G10" s="64" t="s">
-        <v>33</v>
-      </c>
-      <c r="H10" s="66"/>
-      <c r="I10" s="65"/>
+      <c r="F10" s="55"/>
+      <c r="G10" s="54" t="s">
+        <v>34</v>
+      </c>
+      <c r="H10" s="56"/>
+      <c r="I10" s="55"/>
       <c r="J10" s="10"/>
     </row>
     <row r="11" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3092,31 +3092,31 @@
       <c r="F12" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="67" t="s">
+      <c r="G12" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="H12" s="68"/>
-      <c r="I12" s="69"/>
+      <c r="H12" s="60"/>
+      <c r="I12" s="61"/>
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:12" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
-      <c r="B13" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" s="46"/>
-      <c r="D13" s="47" t="s">
+      <c r="B13" s="63" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="64"/>
+      <c r="D13" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="48"/>
+      <c r="E13" s="66"/>
       <c r="F13" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="49" t="s">
+      <c r="G13" s="67" t="s">
         <v>37</v>
       </c>
-      <c r="H13" s="50"/>
-      <c r="I13" s="51"/>
+      <c r="H13" s="68"/>
+      <c r="I13" s="69"/>
       <c r="J13" s="10"/>
     </row>
     <row r="14" spans="1:12" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3143,10 +3143,10 @@
       <c r="E15" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="52" t="s">
+      <c r="F15" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="G15" s="53"/>
+      <c r="G15" s="71"/>
       <c r="H15" s="11"/>
       <c r="I15" s="16" t="s">
         <v>16</v>
@@ -3166,10 +3166,10 @@
       <c r="E16" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="54" t="s">
+      <c r="F16" s="72" t="s">
         <v>42</v>
       </c>
-      <c r="G16" s="55"/>
+      <c r="G16" s="73"/>
       <c r="H16" s="11"/>
       <c r="I16" s="20" t="s">
         <v>43</v>
@@ -3177,16 +3177,16 @@
       <c r="L16" s="4"/>
     </row>
     <row r="17" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="56" t="s">
+      <c r="B17" s="74" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="56"/>
-      <c r="D17" s="56"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="56"/>
-      <c r="I17" s="56"/>
+      <c r="C17" s="74"/>
+      <c r="D17" s="74"/>
+      <c r="E17" s="74"/>
+      <c r="F17" s="74"/>
+      <c r="G17" s="74"/>
+      <c r="H17" s="74"/>
+      <c r="I17" s="74"/>
       <c r="L17" s="21"/>
       <c r="M17" s="21"/>
       <c r="N17" s="21"/>
@@ -3231,8 +3231,8 @@
       <c r="E19" s="28"/>
       <c r="F19" s="29"/>
       <c r="G19" s="29"/>
-      <c r="H19" s="54"/>
-      <c r="I19" s="55"/>
+      <c r="H19" s="72"/>
+      <c r="I19" s="73"/>
       <c r="L19" s="21"/>
       <c r="M19" s="22"/>
       <c r="N19" s="22"/>
@@ -3249,8 +3249,8 @@
       <c r="E20" s="28"/>
       <c r="F20" s="29"/>
       <c r="G20" s="29"/>
-      <c r="H20" s="54"/>
-      <c r="I20" s="55"/>
+      <c r="H20" s="72"/>
+      <c r="I20" s="73"/>
       <c r="L20" s="21"/>
       <c r="M20" s="22"/>
       <c r="N20" s="21"/>
@@ -3278,12 +3278,12 @@
       <c r="B22" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="59"/>
-      <c r="D22" s="59"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="59"/>
-      <c r="G22" s="59"/>
-      <c r="H22" s="59"/>
+      <c r="C22" s="75"/>
+      <c r="D22" s="75"/>
+      <c r="E22" s="75"/>
+      <c r="F22" s="75"/>
+      <c r="G22" s="75"/>
+      <c r="H22" s="75"/>
       <c r="I22" s="58"/>
       <c r="L22" s="34"/>
       <c r="M22" s="22"/>
@@ -3312,16 +3312,16 @@
       <c r="Q23" s="22"/>
     </row>
     <row r="24" spans="1:17" ht="34.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="60" t="s">
+      <c r="B24" s="76" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
-      <c r="G24" s="60"/>
-      <c r="H24" s="60"/>
-      <c r="I24" s="60"/>
+      <c r="C24" s="76"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="76"/>
+      <c r="G24" s="76"/>
+      <c r="H24" s="76"/>
+      <c r="I24" s="76"/>
     </row>
     <row r="25" spans="1:17" ht="34.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="41"/>
@@ -3364,16 +3364,16 @@
       <c r="I28" s="41"/>
     </row>
     <row r="29" spans="1:17" ht="34.15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="44" t="s">
+      <c r="B29" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="44"/>
-      <c r="D29" s="44"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="44"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="44"/>
-      <c r="I29" s="44"/>
+      <c r="C29" s="62"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="62"/>
+      <c r="G29" s="62"/>
+      <c r="H29" s="62"/>
+      <c r="I29" s="62"/>
     </row>
     <row r="30" spans="1:17" ht="102.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
@@ -3399,18 +3399,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B7:I7"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:I12"/>
     <mergeCell ref="B29:I29"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="D13:E13"/>
@@ -3423,6 +3411,18 @@
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="B22:I22"/>
     <mergeCell ref="B24:I24"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="B7:I7"/>
+    <mergeCell ref="B8:I8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="G9:I9"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.27559055118110237" right="0.31496062992125984" top="0.59055118110236227" bottom="0.47244094488188981" header="0.62992125984251968" footer="0.43307086614173229"/>

</xml_diff>